<commit_message>
Ydelsesbeskrivelse og opdaterede punkter i honoraroverslag, Hjerlesvej
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ordoCcUEbJneMEHBU2jJd
</commit_message>
<xml_diff>
--- a/energi/projekter/hjerlesvej/tilbud/Honoraroverslag_Hjerlesvej.xlsx
+++ b/energi/projekter/hjerlesvej/tilbud/Honoraroverslag_Hjerlesvej.xlsx
@@ -1869,7 +1869,7 @@
     <row r="24" ht="15.6" customHeight="1">
       <c r="A24" s="73" t="inlineStr">
         <is>
-          <t>Funderingsløsning for ny bygning og tilslutning til eksisterende fundamenter</t>
+          <t>Funderingsløsninger for udbedring af sætninger</t>
         </is>
       </c>
       <c r="B24" s="32" t="n"/>
@@ -1878,7 +1878,7 @@
     <row r="25" ht="15.6" customHeight="1">
       <c r="A25" s="73" t="inlineStr">
         <is>
-          <t>Principper for evt. forstærkning af eksisterende fundamenter</t>
+          <t>Funderingsløsning for ny bygning og tilslutning til eksisterende fundamenter</t>
         </is>
       </c>
       <c r="B25" s="32" t="n"/>
@@ -1940,7 +1940,7 @@
     <row r="31" ht="15.6" customHeight="1">
       <c r="A31" s="73" t="inlineStr">
         <is>
-          <t>Opdateret statik: bjælker, vægge og søjler</t>
+          <t>Stabilitet</t>
         </is>
       </c>
       <c r="B31" s="32" t="n"/>
@@ -1951,7 +1951,7 @@
     <row r="32" ht="15.6" customHeight="1">
       <c r="A32" s="73" t="inlineStr">
         <is>
-          <t>Nye åbninger og tilslutning til ny bygning</t>
+          <t>Bjælker og søjler</t>
         </is>
       </c>
       <c r="B32" s="32" t="n"/>
@@ -1962,7 +1962,7 @@
     <row r="33" ht="15.6" customHeight="1">
       <c r="A33" s="73" t="inlineStr">
         <is>
-          <t>Stabilitet ved ændrede vægge</t>
+          <t>Deformationer</t>
         </is>
       </c>
       <c r="B33" s="32" t="n"/>
@@ -1971,7 +1971,7 @@
     <row r="34" ht="15.6" customHeight="1">
       <c r="A34" s="73" t="inlineStr">
         <is>
-          <t>Beregninger og tegninger for ændringer</t>
+          <t>Nye åbninger og tilslutning til ny bygning</t>
         </is>
       </c>
       <c r="B34" s="277" t="n"/>
@@ -2022,7 +2022,7 @@
     <row r="39" ht="15.6" customHeight="1">
       <c r="A39" s="73" t="inlineStr">
         <is>
-          <t>Ny konstruktion: bjælker, vægge og søjler</t>
+          <t>Ny konstruktion: fundering</t>
         </is>
       </c>
       <c r="B39" s="32" t="n"/>
@@ -2031,7 +2031,7 @@
     <row r="40" ht="15.6" customHeight="1">
       <c r="A40" s="73" t="inlineStr">
         <is>
-          <t>Stabilitet: vindafstivning og skiver</t>
+          <t>Ny konstruktion: bjælker og søjler</t>
         </is>
       </c>
       <c r="B40" s="32" t="n"/>
@@ -2040,7 +2040,7 @@
     <row r="41" ht="15.6" customHeight="1">
       <c r="A41" s="73" t="inlineStr">
         <is>
-          <t>Fundamenter</t>
+          <t>Ny konstruktion: vægge og stabilitet</t>
         </is>
       </c>
       <c r="B41" s="32" t="n"/>
@@ -2049,7 +2049,7 @@
     <row r="42" ht="15.6" customHeight="1">
       <c r="A42" s="73" t="inlineStr">
         <is>
-          <t>A-frame: vurdering ved nye laster, dobbelthøjt rum og nye gavlåbninger</t>
+          <t>A-frame: vurdering af deformationer ved nye glaspartier</t>
         </is>
       </c>
       <c r="B42" s="32" t="n"/>
@@ -2058,7 +2058,7 @@
     <row r="43" ht="15.6" customHeight="1">
       <c r="A43" s="73" t="inlineStr">
         <is>
-          <t>Kurvede bjælker ved køkken</t>
+          <t>A-frame: vurdering ved nye laster og dobbelthøjt rum</t>
         </is>
       </c>
       <c r="B43" s="32" t="n"/>
@@ -2067,7 +2067,7 @@
     <row r="44" ht="15.6" customHeight="1">
       <c r="A44" s="73" t="inlineStr">
         <is>
-          <t>Samling mellem anneks, ny bygning og A-frame</t>
+          <t>Åbning ved køkken og buede bjælker</t>
         </is>
       </c>
       <c r="B44" s="32" t="n"/>
@@ -2076,7 +2076,7 @@
     <row r="45" ht="15.6" customHeight="1">
       <c r="A45" s="73" t="inlineStr">
         <is>
-          <t>Trappe og repos</t>
+          <t>Flytning af glasfacader</t>
         </is>
       </c>
       <c r="B45" s="32" t="n"/>
@@ -2085,7 +2085,7 @@
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="73" t="inlineStr">
         <is>
-          <t>Konstruktionstegninger (planer, snit, principdetaljer)</t>
+          <t>Samling mellem anneks, ny bygning og A-frame</t>
         </is>
       </c>
       <c r="B46" s="32" t="n"/>
@@ -2094,7 +2094,7 @@
     <row r="47" ht="15.6" customHeight="1">
       <c r="A47" s="73" t="inlineStr">
         <is>
-          <t>Statisk dokumentation: A1 Konstruktionsgrundlag, A2 Statiske beregninger, B1 Statisk projektredegørelse</t>
+          <t>Beregning af trappe og repos</t>
         </is>
       </c>
       <c r="B47" s="277" t="n"/>
@@ -2103,7 +2103,7 @@
     <row r="48" ht="15.6" customHeight="1">
       <c r="A48" s="73" t="inlineStr">
         <is>
-          <t>Indeklima: termisk indeklima, dagslys og varmetabsramme (notat)</t>
+          <t>Konstruktionstegninger og statisk dokumentation (A1, A2, B1)</t>
         </is>
       </c>
       <c r="B48" s="277" t="n"/>
@@ -2112,7 +2112,7 @@
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="73" t="inlineStr">
         <is>
-          <t>Møder og koordinering med arkitekt og entreprenør</t>
+          <t>Indeklima samt møder og koordinering med arkitekt og entreprenør</t>
         </is>
       </c>
       <c r="B49" s="32" t="n"/>

</xml_diff>

<commit_message>
Honoraroverslag: uddybning af hvert punkt under tabellen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ordoCcUEbJneMEHBU2jJd
</commit_message>
<xml_diff>
--- a/energi/projekter/hjerlesvej/tilbud/Honoraroverslag_Hjerlesvej.xlsx
+++ b/energi/projekter/hjerlesvej/tilbud/Honoraroverslag_Hjerlesvej.xlsx
@@ -872,7 +872,7 @@
     <xf numFmtId="0" fontId="16" fillId="8" borderId="0"/>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="280">
+  <cellXfs count="281">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1349,6 +1349,7 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="165" fontId="25" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2174,35 +2175,47 @@
       <c r="B55" s="32" t="n"/>
       <c r="C55" s="32" t="n"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="32" t="n"/>
-      <c r="B56" s="277" t="n"/>
-      <c r="C56" s="277" t="n"/>
-    </row>
-    <row r="57" ht="15.6" customHeight="1">
-      <c r="A57" s="32" t="n"/>
-      <c r="B57" s="277" t="n"/>
-      <c r="C57" s="277" t="n"/>
-    </row>
-    <row r="58" ht="14.25" customHeight="1">
-      <c r="A58" s="32" t="n"/>
-      <c r="B58" s="32" t="n"/>
-      <c r="C58" s="32" t="n"/>
-    </row>
-    <row r="59" ht="14.25" customHeight="1">
-      <c r="A59" s="32" t="n"/>
-      <c r="B59" s="32" t="n"/>
-      <c r="C59" s="32" t="n"/>
-    </row>
-    <row r="60" ht="15.6" customHeight="1">
-      <c r="A60" s="32" t="n"/>
-      <c r="B60" s="32" t="n"/>
-      <c r="C60" s="32" t="n"/>
-    </row>
-    <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="32" t="n"/>
-      <c r="B61" s="277" t="n"/>
-      <c r="C61" s="277" t="n"/>
+    <row r="56" ht="21" customHeight="1">
+      <c r="A56" s="280" t="inlineStr">
+        <is>
+          <t>Uddybning af overslaget</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="55.5" customHeight="1">
+      <c r="A57" s="263" t="inlineStr">
+        <is>
+          <t>Overslaget er delt i tre punkter, som svarer til tabellen ovenfor. Spændet mellem min. og max. afspejler, at der endnu ikke er foretaget besigtigelse eller geoteknisk undersøgelse. Afregning sker i medgået tid inden for rammen, så I kun betaler for de timer, opgaven reelt kræver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="86.7" customHeight="1">
+      <c r="A58" s="263" t="inlineStr">
+        <is>
+          <t>Punkt 1 – Geoteknik og funderingsløsninger (35–50 timer). Der er sætningsskader på den eksisterende bygning, og de skal forstås, før vi kan fundere nyt. Vi besigtiger og registrerer skaderne, laver boreplan, koordinerer med geoteknikeren og gennemgår rapporten. Derefter projekterer vi både udbedring af sætningerne og funderingen af den nye bygning, så nye og gamle fundamenter ikke sætter sig forskelligt. Viser undersøgelsen fast bund i normal dybde, lander vi i den lave ende. Kræver jorden dybere eller særlig fundering, lander vi i den høje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="55.5" customHeight="1">
+      <c r="A59" s="263" t="inlineStr">
+        <is>
+          <t>Punkt 2 – Anneks (30–45 timer). Annekset fra 2001 er godt dokumenteret, og derfor er punktet relativt lille. Vægge ændres, der laves nye åbninger, og bygningen kobles på den nye bygning. Derfor skal stabiliteten, bjælker og søjler samt deformationerne eftervises på ny. Den høje ende dækker, at besigtigelsen viser afvigelser fra tegningerne.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="133.5" customHeight="1">
+      <c r="A60" s="263" t="inlineStr">
+        <is>
+          <t>Punkt 3 – Ny bygning og A-frame (190–240 timer). Dette er projektets største og mest komplekse del og fordeler sig groft således: Ny konstruktion ca. 70–85 timer (laster inkl. snesæk mod A-husets tag, fundering, bjælker, søjler, vægge og stabilitet). A-frame ca. 60–80 timer: Huset fra 1973 har ingen statiske beregninger i byggesagsarkivet, så konstruktionens bæreevne skal fastlægges fra bunden. Dertil kommer vurdering af deformationer ved de nye glaspartier, da store glasflader kun tåler små bevægelser, konsekvensen af det dobbelthøje rum, hvor etagedæk og hanebånd delvist fjernes, åbningen ved køkkenet og de buede bjælker samt flytning af glasfacader og samlingen mellem de tre bygninger. Trappe og repos ca. 5–10 timer. Konstruktionstegninger og statisk dokumentation (A1, A2, B1) ca. 35–45 timer. Indeklima samt møder og koordinering med arkitekt og entreprenør ca. 20 timer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="55.5" customHeight="1">
+      <c r="A61" s="263" t="inlineStr">
+        <is>
+          <t>Sådan holdes timeforbruget nede: Arkitekten leverer tegninger som DWG eller 3D-model, vi får adgang til huset og kryberummet ved besigtigelsen, og glaspartiernes placering og størrelse fastlægges tidligt. Ændringer, der kommer sent i projekteringen, er det, der typisk flytter et projekt mod den høje ende.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15.6" customHeight="1">
       <c r="A62" s="32" t="n"/>
@@ -2807,23 +2820,29 @@
       <c r="C147" s="84" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="22">
+    <mergeCell ref="A90:C90"/>
+    <mergeCell ref="A89:C89"/>
+    <mergeCell ref="A56:C56"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="A95:C95"/>
+    <mergeCell ref="A2:C2"/>
     <mergeCell ref="A76:C76"/>
+    <mergeCell ref="A116:C116"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A91:C91"/>
+    <mergeCell ref="A72:C72"/>
     <mergeCell ref="A68:C68"/>
-    <mergeCell ref="A90:C90"/>
-    <mergeCell ref="A116:C116"/>
+    <mergeCell ref="A93:C93"/>
+    <mergeCell ref="A58:C58"/>
+    <mergeCell ref="A92:C92"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="A73:C73"/>
+    <mergeCell ref="A60:C60"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A93:C93"/>
-    <mergeCell ref="A89:C89"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A92:C92"/>
-    <mergeCell ref="A91:C91"/>
+    <mergeCell ref="A61:C61"/>
     <mergeCell ref="A69:C69"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A95:C95"/>
-    <mergeCell ref="A73:C73"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A72:C72"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="2">
     <dataValidation sqref="B114" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">

</xml_diff>